<commit_message>
Rename to Talent Conversations; full 10-day sample with candidate batches
The product name and tagline (Talent Conversations, Interviews & assessment)
now live in lib/brand.ts and appear in the sidebar, the login page and the
browser tab, replacing HackJudge / Hackathon Judging. The lightning mark is
now a softer star.

The sample covers all ten weekdays from 19 Oct with the nine panel judges:
a day nobody can sit (22 Oct), an afternoon off (26 Oct), partial windows,
and an afternoon that drops below two judges so four interviews have no
panel. Two candidate batches with realistic names fill the schedule: 66,
then 74 more plus 3 moves and 2 unchanged, leaving 9 slots open. Checked
against the real import: 149 interviews with a panel, 140 placed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qkgbu6zx8nSF6qinJQFGfA
</commit_message>
<xml_diff>
--- a/tools/setup-workbook/sample-candidates-batch1.xlsx
+++ b/tools/setup-workbook/sample-candidates-batch1.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -557,7 +557,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Candidate 001</t>
+          <t>Aisha Tan</t>
         </is>
       </c>
       <c r="B2" s="5" t="n">
@@ -570,7 +570,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Candidate 002</t>
+          <t>Benjamin Lee</t>
         </is>
       </c>
       <c r="B3" s="5" t="n">
@@ -583,7 +583,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Candidate 003</t>
+          <t>Chloe Wijaya</t>
         </is>
       </c>
       <c r="B4" s="5" t="n">
@@ -596,7 +596,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Candidate 004</t>
+          <t>Daniel Lim</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
@@ -609,7 +609,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Candidate 005</t>
+          <t>Elena Santoso</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
@@ -622,7 +622,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Candidate 006</t>
+          <t>Farid Teo</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
@@ -635,7 +635,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Candidate 007</t>
+          <t>Grace Rahman</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
@@ -648,7 +648,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Candidate 008</t>
+          <t>Hafiz Chen</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
@@ -661,7 +661,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Candidate 009</t>
+          <t>Ivy Hassan</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
@@ -669,6 +669,747 @@
       </c>
       <c r="C10" s="6" t="n">
         <v>0.4930555555555556</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Jun Wei Ng</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Kavya Ismail</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>0.5972222222222222</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Mei Ling Kumar</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Nathan Goh</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>0.6388888888888888</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Olivia Reyes</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>0.6597222222222222</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Priya Wong</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>0.6736111111111112</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Qistina Pillai</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>0.6875</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Rahul Koh</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>0.7013888888888888</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Sarah Nguyen</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Thanh Ong</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>0.3888888888888889</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Umar Tan</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>0.4027777777777778</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Vanessa Lee</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Wen Hui Wijaya</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>0.4305555555555556</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Yasmin Santoso</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>0.4652777777777778</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Zhi Hao Teo</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>0.4791666666666667</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Aisha Ng</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>0.4930555555555556</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Benjamin Ismail</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Chloe Chua</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>0.5972222222222222</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Daniel Kumar</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>0.6111111111111112</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Elena Goh</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Farid Reyes</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>0.6388888888888888</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Grace Wong</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>0.6597222222222222</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Hafiz Pillai</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C33" s="6" t="n">
+        <v>0.6736111111111112</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Ivy Koh</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C34" s="6" t="n">
+        <v>0.6875</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Kavya Ong</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Liam Tan</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C36" s="6" t="n">
+        <v>0.3888888888888889</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Mei Ling Lee</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C37" s="6" t="n">
+        <v>0.4027777777777778</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Nathan Wijaya</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C38" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Olivia Lim</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C39" s="6" t="n">
+        <v>0.4305555555555556</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Priya Santoso</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C40" s="6" t="n">
+        <v>0.4513888888888889</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Qistina Teo</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C41" s="6" t="n">
+        <v>0.4652777777777778</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Rahul Rahman</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C42" s="6" t="n">
+        <v>0.4791666666666667</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Sarah Chen</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C43" s="6" t="n">
+        <v>0.4930555555555556</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Thanh Hassan</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C44" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Umar Ng</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C45" s="6" t="n">
+        <v>0.5972222222222222</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Wen Hui Chua</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C46" s="6" t="n">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Xavier Kumar</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C47" s="6" t="n">
+        <v>0.6388888888888888</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Yasmin Goh</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C48" s="6" t="n">
+        <v>0.6597222222222222</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Zhi Hao Reyes</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C49" s="6" t="n">
+        <v>0.6736111111111112</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Aisha Nguyen</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C50" s="6" t="n">
+        <v>0.6875</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Benjamin Ong</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C51" s="6" t="n">
+        <v>0.7013888888888888</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Chloe Tan</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C52" s="6" t="n">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Daniel Lee</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C53" s="6" t="n">
+        <v>0.3888888888888889</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Elena Wijaya</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C54" s="6" t="n">
+        <v>0.4027777777777778</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Farid Lim</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C55" s="6" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Grace Santoso</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C56" s="6" t="n">
+        <v>0.4305555555555556</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Ivy Rahman</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C57" s="6" t="n">
+        <v>0.4652777777777778</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>Jun Wei Chen</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C58" s="6" t="n">
+        <v>0.4791666666666667</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>Kavya Hassan</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C59" s="6" t="n">
+        <v>0.4930555555555556</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>Liam Ng</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C60" s="6" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>Mei Ling Ismail</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C61" s="6" t="n">
+        <v>0.5972222222222222</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>Nathan Chua</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C62" s="6" t="n">
+        <v>0.6111111111111112</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>Olivia Kumar</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C63" s="6" t="n">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>Priya Goh</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C64" s="6" t="n">
+        <v>0.6388888888888888</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>Qistina Reyes</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C65" s="6" t="n">
+        <v>0.6597222222222222</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>Rahul Wong</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C66" s="6" t="n">
+        <v>0.6736111111111112</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>Sarah Pillai</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C67" s="6" t="n">
+        <v>0.6875</v>
       </c>
     </row>
   </sheetData>

</xml_diff>